<commit_message>
Fix boom swing scoring and add visual dashboard
</commit_message>
<xml_diff>
--- a/小挖常见工况竞品量化评分.xlsx
+++ b/小挖常见工况竞品量化评分.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,22 +31,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00263746"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -61,11 +52,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,36 +421,29 @@
   </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>产品</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>综合工况评分</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>平均数据覆盖率</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>综合置信等级</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>原表综合评分</t>
         </is>
@@ -475,7 +456,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57.8</v>
+        <v>60.7</v>
       </c>
       <c r="C2" t="n">
         <v>0.973</v>
@@ -496,7 +477,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>57.5</v>
+        <v>59.4</v>
       </c>
       <c r="C3" t="n">
         <v>0.973</v>
@@ -538,7 +519,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>52.2</v>
+        <v>54.1</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
@@ -580,7 +561,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48.1</v>
+        <v>48.9</v>
       </c>
       <c r="C7" t="n">
         <v>0.89</v>
@@ -601,7 +582,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>47</v>
+        <v>48.9</v>
       </c>
       <c r="C8" t="n">
         <v>0.974</v>
@@ -622,7 +603,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>46.1</v>
+        <v>46.5</v>
       </c>
       <c r="C9" t="n">
         <v>0.85</v>
@@ -691,48 +672,39 @@
   </sheetPr>
   <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>工况</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>产品</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>工况得分</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>数据覆盖率</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>置信等级</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>工况权重</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>工况说明</t>
         </is>
@@ -750,7 +722,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.3</v>
+        <v>38.5</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -781,7 +753,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>38</v>
+        <v>48.5</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -843,7 +815,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>45.5</v>
+        <v>56</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -905,7 +877,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>46.8</v>
+        <v>51.4</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -936,7 +908,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28</v>
+        <v>38.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -967,7 +939,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>39.7</v>
+        <v>42</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -2611,84 +2583,69 @@
   </sheetPr>
   <dimension ref="A1:M531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>工况</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>指标/配置</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>产品</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>原始值</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>数据状态</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>单位</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>方向</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>指标得分</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>权重</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>贡献分</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>相关性说明</t>
         </is>
@@ -4072,6 +4029,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -4087,9 +4045,11 @@
           <t>越低越好</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
         <v>0.24</v>
       </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -4495,13 +4455,13 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>6.3</v>
+        <v>64.3</v>
       </c>
       <c r="J32" t="n">
         <v>0.18</v>
       </c>
       <c r="K32" t="n">
-        <v>1.1</v>
+        <v>11.6</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -4510,7 +4470,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4554,13 +4514,13 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>6.3</v>
+        <v>64.3</v>
       </c>
       <c r="J33" t="n">
         <v>0.18</v>
       </c>
       <c r="K33" t="n">
-        <v>1.1</v>
+        <v>11.6</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -4569,7 +4529,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4595,11 +4555,11 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>258</v>
+        <v>130</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>有数据</t>
+          <t>有数据；驾驶室/驾驶棚版本不同不合计，取同一版本较优口径</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4628,7 +4588,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4653,6 +4613,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -4668,9 +4629,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="n">
         <v>0.18</v>
       </c>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -4737,7 +4700,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4781,13 +4744,13 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1.4</v>
+        <v>14.3</v>
       </c>
       <c r="J37" t="n">
         <v>0.18</v>
       </c>
       <c r="K37" t="n">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -4796,7 +4759,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4840,13 +4803,13 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>9.9</v>
+        <v>100</v>
       </c>
       <c r="J38" t="n">
         <v>0.18</v>
       </c>
       <c r="K38" t="n">
-        <v>1.8</v>
+        <v>18</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4855,7 +4818,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4862,13 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>6.3</v>
+        <v>64.3</v>
       </c>
       <c r="J39" t="n">
         <v>0.18</v>
       </c>
       <c r="K39" t="n">
-        <v>1.1</v>
+        <v>11.6</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -4914,7 +4877,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4958,13 +4921,13 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>2.8</v>
+        <v>28.6</v>
       </c>
       <c r="J40" t="n">
         <v>0.18</v>
       </c>
       <c r="K40" t="n">
-        <v>0.5</v>
+        <v>5.1</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -4973,7 +4936,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>贴墙、沟边、障碍物旁作业能力。</t>
+          <t>贴墙、沟边、障碍物旁作业能力；多版本参数按同一版本口径取值，不相加。</t>
         </is>
       </c>
     </row>
@@ -4998,6 +4961,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -5013,9 +4977,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
         <v>0.18</v>
       </c>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -7626,6 +7592,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -7641,9 +7608,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I85" t="inlineStr"/>
       <c r="J85" t="n">
         <v>0.16</v>
       </c>
+      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -7971,6 +7940,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -7986,9 +7956,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I91" t="inlineStr"/>
       <c r="J91" t="n">
         <v>0.16</v>
       </c>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -8139,6 +8111,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -8154,9 +8127,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I94" t="inlineStr"/>
       <c r="J94" t="n">
         <v>0.12</v>
       </c>
+      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -10332,6 +10307,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>未披露</t>
@@ -10347,9 +10323,11 @@
           <t>标配&gt;选配&gt;无；未披露不参与</t>
         </is>
       </c>
+      <c r="I131" t="inlineStr"/>
       <c r="J131" t="n">
         <v>0.08</v>
       </c>
+      <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
           <t>3-4.xlsx 标选配表</t>
@@ -10748,6 +10726,7 @@
           <t>沃尔沃 EC37</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>未披露</t>
@@ -10763,9 +10742,11 @@
           <t>标配&gt;选配&gt;无；未披露不参与</t>
         </is>
       </c>
+      <c r="I138" t="inlineStr"/>
       <c r="J138" t="n">
         <v>0.06</v>
       </c>
+      <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
           <t>3-4.xlsx 标选配表</t>
@@ -10798,6 +10779,7 @@
           <t>现代 HX35AZ</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>未披露</t>
@@ -10813,9 +10795,11 @@
           <t>标配&gt;选配&gt;无；未披露不参与</t>
         </is>
       </c>
+      <c r="I139" t="inlineStr"/>
       <c r="J139" t="n">
         <v>0.06</v>
       </c>
+      <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
           <t>3-4.xlsx 标选配表</t>
@@ -10848,6 +10832,7 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>未披露</t>
@@ -10863,9 +10848,11 @@
           <t>标配&gt;选配&gt;无；未披露不参与</t>
         </is>
       </c>
+      <c r="I140" t="inlineStr"/>
       <c r="J140" t="n">
         <v>0.06</v>
       </c>
+      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>3-4.xlsx 标选配表</t>
@@ -10898,6 +10885,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>未披露</t>
@@ -10913,9 +10901,11 @@
           <t>标配&gt;选配&gt;无；未披露不参与</t>
         </is>
       </c>
+      <c r="I141" t="inlineStr"/>
       <c r="J141" t="n">
         <v>0.06</v>
       </c>
+      <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>
           <t>3-4.xlsx 标选配表</t>
@@ -12895,6 +12885,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -12910,9 +12901,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I175" t="inlineStr"/>
       <c r="J175" t="n">
         <v>0.144</v>
       </c>
+      <c r="K175" t="inlineStr"/>
       <c r="L175" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -13417,6 +13410,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -13432,9 +13426,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I184" t="inlineStr"/>
       <c r="J184" t="n">
         <v>0.09</v>
       </c>
+      <c r="K184" t="inlineStr"/>
       <c r="L184" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -13467,6 +13463,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -13482,9 +13479,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I185" t="inlineStr"/>
       <c r="J185" t="n">
         <v>0.09</v>
       </c>
+      <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -13517,6 +13516,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -13532,9 +13532,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I186" t="inlineStr"/>
       <c r="J186" t="n">
         <v>0.09</v>
       </c>
+      <c r="K186" t="inlineStr"/>
       <c r="L186" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -13567,6 +13569,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -13582,9 +13585,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I187" t="inlineStr"/>
       <c r="J187" t="n">
         <v>0.09</v>
       </c>
+      <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -14030,6 +14035,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -14045,9 +14051,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I195" t="inlineStr"/>
       <c r="J195" t="n">
         <v>0.108</v>
       </c>
+      <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -15142,6 +15150,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -15157,9 +15166,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I214" t="inlineStr"/>
       <c r="J214" t="n">
         <v>0.09</v>
       </c>
+      <c r="K214" t="inlineStr"/>
       <c r="L214" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -16667,6 +16678,7 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -16682,9 +16694,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I240" t="inlineStr"/>
       <c r="J240" t="n">
         <v>0.2</v>
       </c>
+      <c r="K240" t="inlineStr"/>
       <c r="L240" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -16894,6 +16908,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -16909,9 +16924,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I244" t="inlineStr"/>
       <c r="J244" t="n">
         <v>0.14</v>
       </c>
+      <c r="K244" t="inlineStr"/>
       <c r="L244" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17003,6 +17020,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17018,9 +17036,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I246" t="inlineStr"/>
       <c r="J246" t="n">
         <v>0.14</v>
       </c>
+      <c r="K246" t="inlineStr"/>
       <c r="L246" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17053,6 +17073,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17068,9 +17089,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I247" t="inlineStr"/>
       <c r="J247" t="n">
         <v>0.14</v>
       </c>
+      <c r="K247" t="inlineStr"/>
       <c r="L247" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17221,6 +17244,7 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17236,9 +17260,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I250" t="inlineStr"/>
       <c r="J250" t="n">
         <v>0.14</v>
       </c>
+      <c r="K250" t="inlineStr"/>
       <c r="L250" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17448,6 +17474,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17463,9 +17490,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I254" t="inlineStr"/>
       <c r="J254" t="n">
         <v>0.16</v>
       </c>
+      <c r="K254" t="inlineStr"/>
       <c r="L254" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17498,6 +17527,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17513,9 +17543,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I255" t="inlineStr"/>
       <c r="J255" t="n">
         <v>0.16</v>
       </c>
+      <c r="K255" t="inlineStr"/>
       <c r="L255" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17548,6 +17580,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17563,9 +17596,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I256" t="inlineStr"/>
       <c r="J256" t="n">
         <v>0.16</v>
       </c>
+      <c r="K256" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17598,6 +17633,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17613,9 +17649,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I257" t="inlineStr"/>
       <c r="J257" t="n">
         <v>0.16</v>
       </c>
+      <c r="K257" t="inlineStr"/>
       <c r="L257" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17766,6 +17804,7 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17781,9 +17820,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I260" t="inlineStr"/>
       <c r="J260" t="n">
         <v>0.16</v>
       </c>
+      <c r="K260" t="inlineStr"/>
       <c r="L260" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17816,6 +17857,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17831,9 +17873,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I261" t="inlineStr"/>
       <c r="J261" t="n">
         <v>0.16</v>
       </c>
+      <c r="K261" t="inlineStr"/>
       <c r="L261" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -17984,6 +18028,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E264" t="inlineStr"/>
       <c r="F264" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -17999,9 +18044,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I264" t="inlineStr"/>
       <c r="J264" t="n">
         <v>0.12</v>
       </c>
+      <c r="K264" t="inlineStr"/>
       <c r="L264" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18034,6 +18081,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18049,9 +18097,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I265" t="inlineStr"/>
       <c r="J265" t="n">
         <v>0.12</v>
       </c>
+      <c r="K265" t="inlineStr"/>
       <c r="L265" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18084,6 +18134,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18099,9 +18150,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I266" t="inlineStr"/>
       <c r="J266" t="n">
         <v>0.12</v>
       </c>
+      <c r="K266" t="inlineStr"/>
       <c r="L266" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18134,6 +18187,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18149,9 +18203,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I267" t="inlineStr"/>
       <c r="J267" t="n">
         <v>0.12</v>
       </c>
+      <c r="K267" t="inlineStr"/>
       <c r="L267" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18302,6 +18358,7 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr"/>
       <c r="F270" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18317,9 +18374,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I270" t="inlineStr"/>
       <c r="J270" t="n">
         <v>0.12</v>
       </c>
+      <c r="K270" t="inlineStr"/>
       <c r="L270" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18352,6 +18411,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr"/>
       <c r="F271" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18367,9 +18427,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I271" t="inlineStr"/>
       <c r="J271" t="n">
         <v>0.12</v>
       </c>
+      <c r="K271" t="inlineStr"/>
       <c r="L271" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -18579,6 +18641,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr"/>
       <c r="F275" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -18594,9 +18657,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I275" t="inlineStr"/>
       <c r="J275" t="n">
         <v>0.12</v>
       </c>
+      <c r="K275" t="inlineStr"/>
       <c r="L275" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -19101,6 +19166,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E284" t="inlineStr"/>
       <c r="F284" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -19116,9 +19182,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I284" t="inlineStr"/>
       <c r="J284" t="n">
         <v>0.1</v>
       </c>
+      <c r="K284" t="inlineStr"/>
       <c r="L284" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -19151,6 +19219,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -19166,9 +19235,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I285" t="inlineStr"/>
       <c r="J285" t="n">
         <v>0.1</v>
       </c>
+      <c r="K285" t="inlineStr"/>
       <c r="L285" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -19201,6 +19272,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -19216,9 +19288,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I286" t="inlineStr"/>
       <c r="J286" t="n">
         <v>0.1</v>
       </c>
+      <c r="K286" t="inlineStr"/>
       <c r="L286" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -19251,6 +19325,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -19266,9 +19341,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I287" t="inlineStr"/>
       <c r="J287" t="n">
         <v>0.1</v>
       </c>
+      <c r="K287" t="inlineStr"/>
       <c r="L287" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -21465,6 +21542,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E324" t="inlineStr"/>
       <c r="F324" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -21480,9 +21558,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I324" t="inlineStr"/>
       <c r="J324" t="n">
         <v>0.1273</v>
       </c>
+      <c r="K324" t="inlineStr"/>
       <c r="L324" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -21515,6 +21595,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E325" t="inlineStr"/>
       <c r="F325" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -21530,9 +21611,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I325" t="inlineStr"/>
       <c r="J325" t="n">
         <v>0.1273</v>
       </c>
+      <c r="K325" t="inlineStr"/>
       <c r="L325" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22037,6 +22120,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E334" t="inlineStr"/>
       <c r="F334" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22052,9 +22136,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I334" t="inlineStr"/>
       <c r="J334" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K334" t="inlineStr"/>
       <c r="L334" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22087,6 +22173,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22102,9 +22189,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I335" t="inlineStr"/>
       <c r="J335" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K335" t="inlineStr"/>
       <c r="L335" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22137,6 +22226,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E336" t="inlineStr"/>
       <c r="F336" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22152,9 +22242,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I336" t="inlineStr"/>
       <c r="J336" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K336" t="inlineStr"/>
       <c r="L336" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22187,6 +22279,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E337" t="inlineStr"/>
       <c r="F337" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22202,9 +22295,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I337" t="inlineStr"/>
       <c r="J337" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K337" t="inlineStr"/>
       <c r="L337" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22237,6 +22332,7 @@
           <t>沃尔沃 EC37</t>
         </is>
       </c>
+      <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22252,9 +22348,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I338" t="inlineStr"/>
       <c r="J338" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K338" t="inlineStr"/>
       <c r="L338" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -22641,6 +22739,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E345" t="inlineStr"/>
       <c r="F345" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -22656,9 +22755,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I345" t="inlineStr"/>
       <c r="J345" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K345" t="inlineStr"/>
       <c r="L345" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -23222,6 +23323,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -23237,9 +23339,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I355" t="inlineStr"/>
       <c r="J355" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K355" t="inlineStr"/>
       <c r="L355" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -23272,6 +23376,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E356" t="inlineStr"/>
       <c r="F356" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -23287,9 +23392,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I356" t="inlineStr"/>
       <c r="J356" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K356" t="inlineStr"/>
       <c r="L356" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -23322,6 +23429,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -23337,9 +23445,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I357" t="inlineStr"/>
       <c r="J357" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K357" t="inlineStr"/>
       <c r="L357" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -23608,6 +23718,7 @@
           <t>XCMG XE35U</t>
         </is>
       </c>
+      <c r="E362" t="inlineStr"/>
       <c r="F362" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -23623,9 +23734,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I362" t="inlineStr"/>
       <c r="J362" t="n">
         <v>0.1455</v>
       </c>
+      <c r="K362" t="inlineStr"/>
       <c r="L362" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -23835,6 +23948,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E366" t="inlineStr"/>
       <c r="F366" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -23850,9 +23964,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I366" t="inlineStr"/>
       <c r="J366" t="n">
         <v>0.1455</v>
       </c>
+      <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24121,6 +24237,7 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="E371" t="inlineStr"/>
       <c r="F371" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24136,9 +24253,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I371" t="inlineStr"/>
       <c r="J371" t="n">
         <v>0.1455</v>
       </c>
+      <c r="K371" t="inlineStr"/>
       <c r="L371" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24289,6 +24408,7 @@
           <t>迪尔 35P</t>
         </is>
       </c>
+      <c r="E374" t="inlineStr"/>
       <c r="F374" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24304,9 +24424,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I374" t="inlineStr"/>
       <c r="J374" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K374" t="inlineStr"/>
       <c r="L374" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24339,6 +24461,7 @@
           <t>山猫 E35</t>
         </is>
       </c>
+      <c r="E375" t="inlineStr"/>
       <c r="F375" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24354,9 +24477,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I375" t="inlineStr"/>
       <c r="J375" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K375" t="inlineStr"/>
       <c r="L375" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24389,6 +24514,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E376" t="inlineStr"/>
       <c r="F376" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24404,9 +24530,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I376" t="inlineStr"/>
       <c r="J376" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24439,6 +24567,7 @@
           <t>久保田 KX033</t>
         </is>
       </c>
+      <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24454,9 +24583,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I377" t="inlineStr"/>
       <c r="J377" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K377" t="inlineStr"/>
       <c r="L377" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24548,6 +24679,7 @@
           <t>现代 HX35AZ</t>
         </is>
       </c>
+      <c r="E379" t="inlineStr"/>
       <c r="F379" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24563,9 +24695,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I379" t="inlineStr"/>
       <c r="J379" t="n">
         <v>0.09089999999999999</v>
       </c>
+      <c r="K379" t="inlineStr"/>
       <c r="L379" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -24952,6 +25086,7 @@
           <t>久保田 U35</t>
         </is>
       </c>
+      <c r="E386" t="inlineStr"/>
       <c r="F386" t="inlineStr">
         <is>
           <t>缺失/未披露</t>
@@ -24967,9 +25102,11 @@
           <t>越高越好</t>
         </is>
       </c>
+      <c r="I386" t="inlineStr"/>
       <c r="J386" t="n">
         <v>0.1273</v>
       </c>
+      <c r="K386" t="inlineStr"/>
       <c r="L386" t="inlineStr">
         <is>
           <t>3-4.xlsx 参数表</t>
@@ -33730,72 +33867,59 @@
   </sheetPr>
   <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>工况</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>配置</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>产品</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>配置状态</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>数据状态</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>配置得分</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>权重</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>贡献分</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>计分规则</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>对工况影响</t>
         </is>
@@ -35298,14 +35422,17 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="n">
         <v>0.08</v>
       </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>标配=100，选配=60，无配置=0，未披露不参与评分</t>
@@ -35644,14 +35771,17 @@
           <t>沃尔沃 EC37</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
         <v>0.06</v>
       </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>标配=100，选配=60，无配置=0，未披露不参与评分</t>
@@ -35684,14 +35814,17 @@
           <t>现代 HX35AZ</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
         <v>0.06</v>
       </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>标配=100，选配=60，无配置=0，未披露不参与评分</t>
@@ -35724,14 +35857,17 @@
           <t>斗山 DX35Z-7</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
         <v>0.06</v>
       </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>标配=100，选配=60，无配置=0，未披露不参与评分</t>
@@ -35764,14 +35900,17 @@
           <t>三一 SY35U</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
         <v>0.06</v>
       </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>标配=100，选配=60，无配置=0，未披露不参与评分</t>
@@ -41412,36 +41551,29 @@
   </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>工况</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>配置贡献第一</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>第一配置贡献分</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>XCMG配置贡献分</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>XCMG配置排名</t>
         </is>
@@ -41586,36 +41718,29 @@
   </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>工况</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>权重</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>强相关指标</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>指标权重合计</t>
         </is>
@@ -41772,18 +41897,14 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>

</xml_diff>